<commit_message>
fix: feat: expand HireSphere interview workflow features
- add bundled interview package service and UI
- add candidate submission annotation workflow
- add structured evaluation reports
- add backend fallback routes for new services
- update candidate and interviewer dashboard navigation
- add README documentation for new features
</commit_message>
<xml_diff>
--- a/doc/Tasks.xlsx
+++ b/doc/Tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SLIIT\hiresphere-cloud-assignment\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70C616DB-5D18-49D3-8445-8778837F4659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{690BD6F0-71F2-483B-BFDF-07F6C3ADAF0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
   <si>
     <t>Candidates</t>
   </si>
@@ -73,13 +73,31 @@
   </si>
   <si>
     <t>Offer bundled interview packages</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Functions</t>
+  </si>
+  <si>
+    <t>Remark</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -87,16 +105,48 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -104,14 +154,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Bad" xfId="1" builtinId="27"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -390,90 +464,228 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="57.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="57.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
+      <c r="D2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="4"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+      <c r="B3" s="2"/>
+      <c r="C3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="4"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
+      <c r="B4" s="2"/>
+      <c r="C4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="5"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+      <c r="B5" s="2"/>
+      <c r="C5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="5"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
+      <c r="B6" s="2"/>
+      <c r="C6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="5"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
+      <c r="B7" s="2"/>
+      <c r="C7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B8" s="2"/>
+      <c r="C8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="5"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
+      <c r="D9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
+      <c r="D10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="4"/>
+      <c r="F10" s="5"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
+      <c r="D11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="4"/>
+      <c r="F11" s="5"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
+      <c r="D12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="4"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
+      <c r="D13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="4"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
+      <c r="D14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="4"/>
+      <c r="F14" s="5"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="D15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" s="4"/>
+      <c r="F15" s="5"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:B8"/>
+    <mergeCell ref="B9:B15"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>